<commit_message>
fix excel and totales
</commit_message>
<xml_diff>
--- a/admin/presupuesto/TEMPLATE_PRESUPUESTO.xlsx
+++ b/admin/presupuesto/TEMPLATE_PRESUPUESTO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de10c3edaa7a32bb/SOILTECH - NUBE/WEB_ST/SOILTECH_WEB/admin/presupuesto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2925800-487E-47A9-9872-382DE5D2ADD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C2925800-487E-47A9-9872-382DE5D2ADD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EFC6114-7614-4A2B-B880-E8A900D948E2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUPUESTOS" sheetId="1" r:id="rId1"/>
@@ -1053,34 +1053,10 @@
   <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1136,7 +1112,6 @@
     <xf numFmtId="164" fontId="2" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="2" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="10" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1164,11 +1139,36 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1447,377 +1447,337 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="87" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="16">
-        <v>6500</v>
-      </c>
-      <c r="E4" s="17" t="s">
+      <c r="C4" s="5"/>
+      <c r="E4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="18">
-        <v>0.1</v>
-      </c>
-      <c r="E5" s="17" t="s">
+      <c r="C5" s="6"/>
+      <c r="E5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="18">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="C6" s="6"/>
+      <c r="E6" s="2" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="18">
-        <v>0.5</v>
-      </c>
-      <c r="E7" s="17" t="s">
+      <c r="C7" s="6"/>
+      <c r="E7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="18">
-        <v>0.5</v>
-      </c>
-      <c r="E8" s="17" t="s">
+      <c r="C8" s="6"/>
+      <c r="E8" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="15"/>
-      <c r="C9" s="19"/>
-      <c r="E9" s="17"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="7"/>
+      <c r="E9" s="2"/>
     </row>
     <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="3"/>
+      <c r="B11" s="88" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="16">
-        <v>11</v>
-      </c>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="16">
-        <v>3</v>
-      </c>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="16">
-        <v>11</v>
-      </c>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="16">
-        <v>1</v>
-      </c>
+      <c r="C16" s="5"/>
     </row>
     <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="9">
         <f>C13*C14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="9">
+        <f>C15*C16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="10">
+        <f>C17+C18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="11">
+        <f>IF(C13=0,0,C20/C13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="88" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="88"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="E24" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="E25" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="E26" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="E27" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="E28" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="12"/>
+      <c r="E29" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="21">
-        <f>C15*C16</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="22">
-        <f>C17+C18</f>
+    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="E30" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" s="9">
+        <f>110*C4</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="E32" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="E33" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="E34" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="88" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="16">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="23">
-        <f>IF(C13=0,0,C20/C13)</f>
-        <v>181.81818181818181</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14"/>
-      <c r="B23" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-    </row>
-    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="16">
-        <v>2</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="16">
-        <v>4</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="16">
-        <v>5</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="16">
-        <v>350</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="16">
-        <v>2</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="24">
-        <v>12</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C30" s="16">
-        <v>9000</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="21">
-        <f>110*C4</f>
-        <v>715000</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="16">
-        <v>4</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="C33" s="16">
-        <v>100000</v>
-      </c>
-      <c r="E33" s="17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="16">
-        <v>100000</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="14"/>
-      <c r="B36" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
+      <c r="C36" s="88"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
     </row>
     <row r="37" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C37" s="25">
+      <c r="C37" s="13">
         <f>C29*(C27/100)</f>
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="25">
+      <c r="C38" s="13">
         <f>C37*1.2</f>
-        <v>50.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="15" t="s">
+      <c r="B39" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="26">
+      <c r="C39" s="14">
         <f>C38*C28*C30*C24</f>
-        <v>1814400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="15" t="s">
+      <c r="B40" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C40" s="26">
+      <c r="C40" s="14">
         <f>C31*C25*C24</f>
-        <v>5720000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="15" t="s">
+      <c r="B41" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C41" s="26">
+      <c r="C41" s="14">
         <f>C33*C32*C26</f>
-        <v>2000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="15" t="s">
+      <c r="B42" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="14">
         <f>C34*C32*C26</f>
-        <v>2000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="15" t="s">
+      <c r="B44" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C44" s="27">
+      <c r="C44" s="15">
         <f>C7+C8</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1854,865 +1814,786 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="92" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I3" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="16" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="17"/>
+      <c r="B4" s="91" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="91"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="16">
-        <v>1</v>
-      </c>
-      <c r="E5" s="30" t="s">
+      <c r="D5" s="5"/>
+      <c r="E5" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="F5" s="31"/>
-      <c r="G5" s="16">
-        <v>1500000</v>
-      </c>
-      <c r="H5" s="32">
+      <c r="F5" s="19"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="20">
         <f>G5*SUPUESTOS!C13</f>
-        <v>16500000</v>
-      </c>
-      <c r="I5" s="33">
+        <v>0</v>
+      </c>
+      <c r="I5" s="21" t="e">
         <f>H5/SUPUESTOS!$C$4</f>
-        <v>2538.4615384615386</v>
-      </c>
-      <c r="J5" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J5" s="22"/>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="16">
-        <v>1</v>
-      </c>
-      <c r="E6" s="30" t="s">
+      <c r="D6" s="5"/>
+      <c r="E6" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F6" s="16">
-        <v>1</v>
-      </c>
-      <c r="G6" s="16">
-        <v>5000000</v>
-      </c>
-      <c r="H6" s="35">
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="23">
         <f t="shared" ref="H6:H11" si="0">D6*F6*G6</f>
-        <v>5000000</v>
-      </c>
-      <c r="I6" s="33">
+        <v>0</v>
+      </c>
+      <c r="I6" s="21" t="e">
         <f>H6/SUPUESTOS!$C$4</f>
-        <v>769.23076923076928</v>
-      </c>
-      <c r="J6" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J6" s="22"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="16">
-        <v>1</v>
-      </c>
-      <c r="E7" s="30" t="s">
+      <c r="D7" s="5"/>
+      <c r="E7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="16">
-        <v>1</v>
-      </c>
-      <c r="G7" s="16">
-        <v>2000000</v>
-      </c>
-      <c r="H7" s="35">
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="23">
         <f t="shared" si="0"/>
-        <v>2000000</v>
-      </c>
-      <c r="I7" s="33">
+        <v>0</v>
+      </c>
+      <c r="I7" s="21" t="e">
         <f>H7/SUPUESTOS!$C$4</f>
-        <v>307.69230769230768</v>
-      </c>
-      <c r="J7" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J7" s="22"/>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="D8" s="16">
-        <v>0</v>
-      </c>
-      <c r="E8" s="30" t="s">
+      <c r="D8" s="5"/>
+      <c r="E8" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="16">
-        <v>0</v>
-      </c>
-      <c r="G8" s="16">
-        <v>0</v>
-      </c>
-      <c r="H8" s="35">
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I8" s="33">
+      <c r="I8" s="21" t="e">
         <f>H8/SUPUESTOS!$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J8" s="22"/>
     </row>
     <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="16">
-        <v>1</v>
-      </c>
-      <c r="E9" s="30" t="s">
+      <c r="D9" s="5"/>
+      <c r="E9" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F9" s="16">
-        <v>1</v>
-      </c>
-      <c r="G9" s="16">
-        <v>600000</v>
-      </c>
-      <c r="H9" s="35">
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="23">
         <f t="shared" si="0"/>
-        <v>600000</v>
-      </c>
-      <c r="I9" s="33">
+        <v>0</v>
+      </c>
+      <c r="I9" s="21" t="e">
         <f>H9/SUPUESTOS!$C$4</f>
-        <v>92.307692307692307</v>
-      </c>
-      <c r="J9" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J9" s="22"/>
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D10" s="16">
-        <v>1</v>
-      </c>
-      <c r="E10" s="30" t="s">
+      <c r="D10" s="5"/>
+      <c r="E10" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="16">
-        <v>1</v>
-      </c>
-      <c r="G10" s="16">
-        <v>600000</v>
-      </c>
-      <c r="H10" s="35">
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="23">
         <f t="shared" si="0"/>
-        <v>600000</v>
-      </c>
-      <c r="I10" s="33">
+        <v>0</v>
+      </c>
+      <c r="I10" s="21" t="e">
         <f>H10/SUPUESTOS!$C$4</f>
-        <v>92.307692307692307</v>
-      </c>
-      <c r="J10" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J10" s="22"/>
     </row>
     <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="16">
-        <v>0</v>
-      </c>
-      <c r="E11" s="30" t="s">
+      <c r="D11" s="5"/>
+      <c r="E11" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="16">
-        <v>0</v>
-      </c>
-      <c r="G11" s="16">
-        <v>0</v>
-      </c>
-      <c r="H11" s="35">
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="21" t="e">
         <f>H11/SUPUESTOS!$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="34"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J11" s="22"/>
     </row>
     <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="36"/>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="24"/>
+      <c r="B12" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="37">
+      <c r="C12" s="89"/>
+      <c r="D12" s="89"/>
+      <c r="E12" s="89"/>
+      <c r="F12" s="89"/>
+      <c r="G12" s="89"/>
+      <c r="H12" s="25">
         <f>SUM(H5:H11)</f>
-        <v>24700000</v>
-      </c>
-      <c r="I12" s="38">
+        <v>0</v>
+      </c>
+      <c r="I12" s="26" t="e">
         <f>H12/SUPUESTOS!$C$4</f>
-        <v>3800</v>
-      </c>
-      <c r="J12" s="39">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J12" s="27">
         <f>IF(H$35=0,0,H12/H$35)</f>
-        <v>0.63239357126276174</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="29"/>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="17"/>
+      <c r="B13" s="91" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
+      <c r="C13" s="91"/>
+      <c r="D13" s="91"/>
+      <c r="E13" s="91"/>
+      <c r="F13" s="91"/>
+      <c r="G13" s="91"/>
+      <c r="H13" s="91"/>
+      <c r="I13" s="91"/>
+      <c r="J13" s="91"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="40" t="s">
+      <c r="D14" s="29"/>
+      <c r="E14" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42">
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30">
         <f>SUPUESTOS!C40</f>
-        <v>5720000</v>
-      </c>
-      <c r="I14" s="43">
+        <v>0</v>
+      </c>
+      <c r="I14" s="31" t="e">
         <f>H14/SUPUESTOS!$C$4</f>
-        <v>880</v>
-      </c>
-      <c r="J14" s="44"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J14" s="32"/>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="40" t="s">
+      <c r="C15" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="D15" s="41"/>
-      <c r="E15" s="40" t="s">
+      <c r="D15" s="29"/>
+      <c r="E15" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="42">
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30">
         <f>SUPUESTOS!C39</f>
-        <v>1814400</v>
-      </c>
-      <c r="I15" s="43">
+        <v>0</v>
+      </c>
+      <c r="I15" s="31" t="e">
         <f>H15/SUPUESTOS!$C$4</f>
-        <v>279.13846153846151</v>
-      </c>
-      <c r="J15" s="44"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J15" s="32"/>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="36"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="24"/>
+      <c r="B16" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="37">
+      <c r="C16" s="89"/>
+      <c r="D16" s="89"/>
+      <c r="E16" s="89"/>
+      <c r="F16" s="89"/>
+      <c r="G16" s="89"/>
+      <c r="H16" s="25">
         <f>SUM(H14:H15)</f>
-        <v>7534400</v>
-      </c>
-      <c r="I16" s="38">
+        <v>0</v>
+      </c>
+      <c r="I16" s="26" t="e">
         <f>H16/SUPUESTOS!$C$4</f>
-        <v>1159.1384615384616</v>
-      </c>
-      <c r="J16" s="39">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J16" s="27">
         <f>IF(H$35=0,0,H16/H$35)</f>
-        <v>0.1929030819158766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="29"/>
-      <c r="B17" s="10" t="s">
+      <c r="A17" s="17"/>
+      <c r="B17" s="91" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
+      <c r="C17" s="91"/>
+      <c r="D17" s="91"/>
+      <c r="E17" s="91"/>
+      <c r="F17" s="91"/>
+      <c r="G17" s="91"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="91"/>
+      <c r="J17" s="91"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="45" t="s">
+      <c r="A18" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="45" t="s">
+      <c r="C18" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="46"/>
-      <c r="E18" s="45" t="s">
+      <c r="D18" s="34"/>
+      <c r="E18" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="47">
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="35">
         <f>SUPUESTOS!C41</f>
-        <v>2000000</v>
-      </c>
-      <c r="I18" s="48">
+        <v>0</v>
+      </c>
+      <c r="I18" s="36" t="e">
         <f>H18/SUPUESTOS!$C$4</f>
-        <v>307.69230769230768</v>
-      </c>
-      <c r="J18" s="49"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J18" s="37"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="45" t="s">
+      <c r="A19" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="45" t="s">
+      <c r="C19" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="46"/>
-      <c r="E19" s="45" t="s">
+      <c r="D19" s="34"/>
+      <c r="E19" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="47">
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="35">
         <f>SUPUESTOS!C42</f>
-        <v>2000000</v>
-      </c>
-      <c r="I19" s="48">
+        <v>0</v>
+      </c>
+      <c r="I19" s="36" t="e">
         <f>H19/SUPUESTOS!$C$4</f>
-        <v>307.69230769230768</v>
-      </c>
-      <c r="J19" s="49"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J19" s="37"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="36"/>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="24"/>
+      <c r="B20" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="37">
+      <c r="C20" s="89"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="89"/>
+      <c r="G20" s="89"/>
+      <c r="H20" s="25">
         <f>SUM(H18:H19)</f>
-        <v>4000000</v>
-      </c>
-      <c r="I20" s="38">
+        <v>0</v>
+      </c>
+      <c r="I20" s="26" t="e">
         <f>H20/SUPUESTOS!$C$4</f>
-        <v>615.38461538461536</v>
-      </c>
-      <c r="J20" s="39">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J20" s="27">
         <f>IF(H$35=0,0,H20/H$35)</f>
-        <v>0.10241191437453631</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="29"/>
-      <c r="B21" s="10" t="s">
+      <c r="A21" s="17"/>
+      <c r="B21" s="91" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
+      <c r="C21" s="91"/>
+      <c r="D21" s="91"/>
+      <c r="E21" s="91"/>
+      <c r="F21" s="91"/>
+      <c r="G21" s="91"/>
+      <c r="H21" s="91"/>
+      <c r="I21" s="91"/>
+      <c r="J21" s="91"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="50" t="s">
+      <c r="B22" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="50" t="s">
+      <c r="C22" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="16">
-        <v>2</v>
-      </c>
-      <c r="E22" s="50" t="s">
+      <c r="D22" s="5"/>
+      <c r="E22" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="F22" s="16">
-        <v>1</v>
-      </c>
-      <c r="G22" s="51"/>
-      <c r="H22" s="52">
+      <c r="F22" s="5"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="40">
         <f>D22*F22*Equipos!E2</f>
-        <v>208000</v>
-      </c>
-      <c r="I22" s="53">
+        <v>0</v>
+      </c>
+      <c r="I22" s="41" t="e">
         <f>H22/SUPUESTOS!$C$4</f>
-        <v>32</v>
-      </c>
-      <c r="J22" s="54"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J22" s="42"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="B23" s="50" t="s">
+      <c r="B23" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="D23" s="16">
-        <v>1</v>
-      </c>
-      <c r="E23" s="50" t="s">
+      <c r="D23" s="5"/>
+      <c r="E23" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="16">
-        <v>8</v>
-      </c>
-      <c r="G23" s="51"/>
-      <c r="H23" s="52">
+      <c r="F23" s="5"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="40">
         <f>D23*F23*Equipos!E3</f>
-        <v>1066666.6666666667</v>
-      </c>
-      <c r="I23" s="53">
+        <v>0</v>
+      </c>
+      <c r="I23" s="41" t="e">
         <f>H23/SUPUESTOS!$C$4</f>
-        <v>164.10256410256412</v>
-      </c>
-      <c r="J23" s="54"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J23" s="42"/>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="B24" s="50" t="s">
+      <c r="B24" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="50" t="s">
+      <c r="C24" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="D24" s="16">
-        <v>0</v>
-      </c>
-      <c r="E24" s="50" t="s">
+      <c r="D24" s="5"/>
+      <c r="E24" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="F24" s="16">
-        <v>0</v>
-      </c>
-      <c r="G24" s="16">
-        <v>40000</v>
-      </c>
-      <c r="H24" s="55">
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="43">
         <f>D24*F24*G24</f>
         <v>0</v>
       </c>
-      <c r="I24" s="53">
+      <c r="I24" s="41" t="e">
         <f>H24/SUPUESTOS!$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="54"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J24" s="42"/>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="50" t="s">
+      <c r="C25" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="D25" s="16">
-        <v>1</v>
-      </c>
-      <c r="E25" s="50" t="s">
+      <c r="D25" s="5"/>
+      <c r="E25" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="16">
-        <v>8</v>
-      </c>
-      <c r="G25" s="51"/>
-      <c r="H25" s="52">
+      <c r="F25" s="5"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40">
         <f>D25*F25*Equipos!E4</f>
-        <v>400000</v>
-      </c>
-      <c r="I25" s="53">
+        <v>0</v>
+      </c>
+      <c r="I25" s="41" t="e">
         <f>H25/SUPUESTOS!$C$4</f>
-        <v>61.53846153846154</v>
-      </c>
-      <c r="J25" s="54"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J25" s="42"/>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="50" t="s">
+      <c r="C26" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="D26" s="16">
-        <v>1</v>
-      </c>
-      <c r="E26" s="50" t="s">
+      <c r="D26" s="5"/>
+      <c r="E26" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="16">
-        <v>8</v>
-      </c>
-      <c r="G26" s="51"/>
-      <c r="H26" s="52">
+      <c r="F26" s="5"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="40">
         <f>D26*F26*Equipos!E5</f>
-        <v>488888.88888888888</v>
-      </c>
-      <c r="I26" s="53">
+        <v>0</v>
+      </c>
+      <c r="I26" s="41" t="e">
         <f>H26/SUPUESTOS!$C$4</f>
-        <v>75.213675213675216</v>
-      </c>
-      <c r="J26" s="54"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J26" s="42"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
-      <c r="B27" s="9" t="s">
+      <c r="A27" s="24"/>
+      <c r="B27" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="37">
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="89"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="25">
         <f>SUM(H22:H26)</f>
-        <v>2163555.5555555555</v>
-      </c>
-      <c r="I27" s="38">
+        <v>0</v>
+      </c>
+      <c r="I27" s="26" t="e">
         <f>H27/SUPUESTOS!$C$4</f>
-        <v>332.85470085470087</v>
-      </c>
-      <c r="J27" s="39">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J27" s="27">
         <f>IF(H$35=0,0,H27/H$35)</f>
-        <v>5.5393466575026973E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="29"/>
-      <c r="B28" s="10" t="s">
+      <c r="A28" s="17"/>
+      <c r="B28" s="91" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
+      <c r="C28" s="91"/>
+      <c r="D28" s="91"/>
+      <c r="E28" s="91"/>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91"/>
+      <c r="H28" s="91"/>
+      <c r="I28" s="91"/>
+      <c r="J28" s="91"/>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="56" t="s">
+      <c r="A29" s="44" t="s">
         <v>110</v>
       </c>
-      <c r="B29" s="56" t="s">
+      <c r="B29" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="56" t="s">
+      <c r="C29" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="D29" s="16">
-        <v>0</v>
-      </c>
-      <c r="E29" s="56" t="s">
+      <c r="D29" s="5"/>
+      <c r="E29" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="F29" s="16">
-        <v>1</v>
-      </c>
-      <c r="G29" s="16">
-        <v>100000</v>
-      </c>
-      <c r="H29" s="26">
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="14">
         <f>D29*F29*G29</f>
         <v>0</v>
       </c>
-      <c r="I29" s="57">
+      <c r="I29" s="45" t="e">
         <f>H29/SUPUESTOS!$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="J29" s="58"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J29" s="46"/>
     </row>
     <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="56" t="s">
+      <c r="A30" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="B30" s="56" t="s">
+      <c r="B30" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="C30" s="56" t="s">
+      <c r="C30" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="D30" s="16">
-        <v>1</v>
-      </c>
-      <c r="E30" s="56" t="s">
+      <c r="D30" s="5"/>
+      <c r="E30" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="F30" s="16">
-        <v>1</v>
-      </c>
-      <c r="G30" s="59"/>
-      <c r="H30" s="60">
+      <c r="F30" s="5"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="48">
         <f>Materiales!E6</f>
-        <v>380000</v>
-      </c>
-      <c r="I30" s="57">
+        <v>0</v>
+      </c>
+      <c r="I30" s="45" t="e">
         <f>H30/SUPUESTOS!$C$4</f>
-        <v>58.46153846153846</v>
-      </c>
-      <c r="J30" s="58"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J30" s="46"/>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="56" t="s">
+      <c r="A31" s="44" t="s">
         <v>115</v>
       </c>
-      <c r="B31" s="56" t="s">
+      <c r="B31" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="56" t="s">
+      <c r="C31" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="D31" s="16">
-        <v>1</v>
-      </c>
-      <c r="E31" s="56" t="s">
+      <c r="D31" s="5"/>
+      <c r="E31" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="F31" s="16">
-        <v>4</v>
-      </c>
-      <c r="G31" s="16">
-        <v>30000</v>
-      </c>
-      <c r="H31" s="26">
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="14">
         <f>D31*F31*G31</f>
-        <v>120000</v>
-      </c>
-      <c r="I31" s="57">
+        <v>0</v>
+      </c>
+      <c r="I31" s="45" t="e">
         <f>H31/SUPUESTOS!$C$4</f>
-        <v>18.46153846153846</v>
-      </c>
-      <c r="J31" s="58"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J31" s="46"/>
     </row>
     <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="56" t="s">
+      <c r="A32" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="B32" s="56" t="s">
+      <c r="B32" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="C32" s="56" t="s">
+      <c r="C32" s="44" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="16">
-        <v>1</v>
-      </c>
-      <c r="E32" s="56" t="s">
+      <c r="D32" s="5"/>
+      <c r="E32" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="F32" s="16">
-        <v>4</v>
-      </c>
-      <c r="G32" s="16">
-        <v>40000</v>
-      </c>
-      <c r="H32" s="26">
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="14">
         <f>D32*F32*G32</f>
-        <v>160000</v>
-      </c>
-      <c r="I32" s="57">
+        <v>0</v>
+      </c>
+      <c r="I32" s="45" t="e">
         <f>H32/SUPUESTOS!$C$4</f>
-        <v>24.615384615384617</v>
-      </c>
-      <c r="J32" s="58"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J32" s="46"/>
     </row>
     <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="36"/>
-      <c r="B33" s="9" t="s">
+      <c r="A33" s="24"/>
+      <c r="B33" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="37">
+      <c r="C33" s="89"/>
+      <c r="D33" s="89"/>
+      <c r="E33" s="89"/>
+      <c r="F33" s="89"/>
+      <c r="G33" s="89"/>
+      <c r="H33" s="25">
         <f>SUM(H29:H32)</f>
-        <v>660000</v>
-      </c>
-      <c r="I33" s="38">
+        <v>0</v>
+      </c>
+      <c r="I33" s="26" t="e">
         <f>H33/SUPUESTOS!$C$4</f>
-        <v>101.53846153846153</v>
-      </c>
-      <c r="J33" s="39">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J33" s="27">
         <f>IF(H$35=0,0,H33/H$35)</f>
-        <v>1.6897965871798492E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="90" t="s">
         <v>120</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="61">
+      <c r="B35" s="90"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="90"/>
+      <c r="E35" s="90"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="90"/>
+      <c r="H35" s="49">
         <f>H12+H16+H20+H27+H33</f>
-        <v>39057955.555555552</v>
-      </c>
-      <c r="I35" s="62">
+        <v>0</v>
+      </c>
+      <c r="I35" s="50" t="e">
         <f>H35/SUPUESTOS!$C$4</f>
-        <v>6008.9162393162387</v>
-      </c>
-      <c r="J35" s="63">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J35" s="51">
         <f>1</f>
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="B16:G16"/>
     <mergeCell ref="B33:G33"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="B17:J17"/>
@@ -2720,11 +2601,6 @@
     <mergeCell ref="B21:J21"/>
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="B28:J28"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:J13"/>
-    <mergeCell ref="B16:G16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2747,170 +2623,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="93" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="94" t="str">
         <f>CONCATENATE("Calicatas: ",SUPUESTOS!C13," × ",SUPUESTOS!C14," muestras = ",SUPUESTOS!C17," | Barrenadas: ",SUPUESTOS!C15," × ",SUPUESTOS!C16," = ",SUPUESTOS!C18," | Total: ",SUPUESTOS!C19)</f>
-        <v>Calicatas: 11 × 3 muestras = 33 | Barrenadas: 11 × 1 = 11 | Total: 44</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+        <v>Calicatas:  ×  muestras = 0 | Barrenadas:  ×  = 0 | Total: 0</v>
+      </c>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
     </row>
     <row r="4" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="G4" s="16" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="8">
         <v>1</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="52">
         <f>SUPUESTOS!C17</f>
-        <v>33</v>
-      </c>
-      <c r="D5" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E5" s="16">
-        <v>255000</v>
-      </c>
-      <c r="F5" s="21">
+      <c r="E5" s="5"/>
+      <c r="F5" s="9">
         <f>C5*E5</f>
-        <v>8415000</v>
-      </c>
-      <c r="G5" s="65">
+        <v>0</v>
+      </c>
+      <c r="G5" s="53" t="e">
         <f>F5/SUPUESTOS!$C$4</f>
-        <v>1294.6153846153845</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="8">
         <v>2</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="64">
+      <c r="C6" s="52">
         <f>SUPUESTOS!C18</f>
-        <v>11</v>
-      </c>
-      <c r="D6" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E6" s="16">
-        <v>190000</v>
-      </c>
-      <c r="F6" s="21">
+      <c r="E6" s="5"/>
+      <c r="F6" s="9">
         <f>C6*E6</f>
-        <v>2090000</v>
-      </c>
-      <c r="G6" s="65">
+        <v>0</v>
+      </c>
+      <c r="G6" s="53" t="e">
         <f>F6/SUPUESTOS!$C$4</f>
-        <v>321.53846153846155</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
+      <c r="A7" s="8">
         <v>3</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C7" s="64">
+      <c r="C7" s="52">
         <f>SUPUESTOS!C17</f>
-        <v>33</v>
-      </c>
-      <c r="D7" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E7" s="16">
-        <v>55000</v>
-      </c>
-      <c r="F7" s="21">
+      <c r="E7" s="5"/>
+      <c r="F7" s="9">
         <f>C7*E7</f>
-        <v>1815000</v>
-      </c>
-      <c r="G7" s="65">
+        <v>0</v>
+      </c>
+      <c r="G7" s="53" t="e">
         <f>F7/SUPUESTOS!$C$4</f>
-        <v>279.23076923076923</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+      <c r="A8" s="8">
         <v>4</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="C8" s="64">
+      <c r="C8" s="52">
         <f>SUPUESTOS!C19</f>
-        <v>44</v>
-      </c>
-      <c r="D8" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E8" s="16">
-        <v>75000</v>
-      </c>
-      <c r="F8" s="21">
+      <c r="E8" s="5"/>
+      <c r="F8" s="9">
         <f>C8*E8</f>
-        <v>3300000</v>
-      </c>
-      <c r="G8" s="65">
+        <v>0</v>
+      </c>
+      <c r="G8" s="53" t="e">
         <f>F8/SUPUESTOS!$C$4</f>
-        <v>507.69230769230768</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="90" t="s">
         <v>131</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="61">
+      <c r="B10" s="90"/>
+      <c r="C10" s="90"/>
+      <c r="D10" s="90"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="49">
         <f>SUM(F5:F8)</f>
-        <v>15620000</v>
-      </c>
-      <c r="G10" s="62">
+        <v>0</v>
+      </c>
+      <c r="G10" s="50" t="e">
         <f>F10/SUPUESTOS!$C$4</f>
-        <v>2403.0769230769229</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -2940,129 +2808,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="93" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
     </row>
     <row r="3" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="16" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="8">
         <v>1</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="16">
-        <v>1</v>
-      </c>
-      <c r="D4" s="20" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="E4" s="16">
-        <v>1000000</v>
-      </c>
-      <c r="F4" s="21">
+      <c r="E4" s="5"/>
+      <c r="F4" s="9">
         <f>C4*E4</f>
-        <v>1000000</v>
-      </c>
-      <c r="G4" s="65">
+        <v>0</v>
+      </c>
+      <c r="G4" s="53" t="e">
         <f>F4/SUPUESTOS!$C$4</f>
-        <v>153.84615384615384</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="16">
-        <v>2</v>
-      </c>
-      <c r="D5" s="20" t="s">
+      <c r="C5" s="5"/>
+      <c r="D5" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="16">
-        <v>7000000</v>
-      </c>
-      <c r="F5" s="21">
+      <c r="E5" s="5"/>
+      <c r="F5" s="9">
         <f>C5*E5</f>
-        <v>14000000</v>
-      </c>
-      <c r="G5" s="65">
+        <v>0</v>
+      </c>
+      <c r="G5" s="53" t="e">
         <f>F5/SUPUESTOS!$C$4</f>
-        <v>2153.8461538461538</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="8">
         <v>3</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="16">
-        <v>0</v>
-      </c>
-      <c r="D6" s="20" t="s">
+      <c r="C6" s="5"/>
+      <c r="D6" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="E6" s="16">
-        <v>1950000</v>
-      </c>
-      <c r="F6" s="21">
+      <c r="E6" s="5"/>
+      <c r="F6" s="9">
         <f>C6*E6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="65">
+      <c r="G6" s="53" t="e">
         <f>F6/SUPUESTOS!$C$4</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="90" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="61">
+      <c r="B8" s="90"/>
+      <c r="C8" s="90"/>
+      <c r="D8" s="90"/>
+      <c r="E8" s="90"/>
+      <c r="F8" s="49">
         <f>SUM(F4:F6)</f>
-        <v>15000000</v>
-      </c>
-      <c r="G8" s="62">
+        <v>0</v>
+      </c>
+      <c r="G8" s="50" t="e">
         <f>F8/SUPUESTOS!$C$4</f>
-        <v>2307.6923076923076</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -3095,524 +2951,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="84" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="H1" s="4" t="s">
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="H1" s="85" t="s">
         <v>140</v>
       </c>
-      <c r="I1" s="4"/>
+      <c r="I1" s="85"/>
     </row>
     <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="I2" s="21">
+      <c r="I2" s="9" t="e">
         <f>C22</f>
-        <v>88348761.711111113</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="64">
+      <c r="C3" s="52">
         <f>Preparación_campo!H35</f>
-        <v>39057955.555555552</v>
-      </c>
-      <c r="D3" s="65">
+        <v>0</v>
+      </c>
+      <c r="D3" s="53" t="e">
         <f>C3/SUPUESTOS!$C$4</f>
-        <v>6008.9162393162387</v>
-      </c>
-      <c r="E3" s="27">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E3" s="15">
         <f>IF($C$6=0,0,C3/$C$6)</f>
-        <v>0.56054967807449385</v>
-      </c>
-      <c r="F3" s="18">
-        <v>0.6</v>
-      </c>
-      <c r="H3" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="H3" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="I3" s="21">
+      <c r="I3" s="9">
         <f>-Preparación_campo!H35</f>
-        <v>-39057955.555555552</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="8">
         <v>2</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C4" s="64">
+      <c r="C4" s="52">
         <f>Laboratorio!F10</f>
-        <v>15620000</v>
-      </c>
-      <c r="D4" s="65">
+        <v>0</v>
+      </c>
+      <c r="D4" s="53" t="e">
         <f>C4/SUPUESTOS!$C$4</f>
-        <v>2403.0769230769229</v>
-      </c>
-      <c r="E4" s="27">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E4" s="15">
         <f>IF($C$6=0,0,C4/$C$6)</f>
-        <v>0.22417420079936012</v>
-      </c>
-      <c r="F4" s="18">
-        <v>0.15</v>
-      </c>
-      <c r="H4" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="H4" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="I4" s="21">
+      <c r="I4" s="9">
         <f>-Laboratorio!F10</f>
-        <v>-15620000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="8">
         <v>3</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="52">
         <f>Informe_final!F8</f>
-        <v>15000000</v>
-      </c>
-      <c r="D5" s="65">
+        <v>0</v>
+      </c>
+      <c r="D5" s="53" t="e">
         <f>C5/SUPUESTOS!$C$4</f>
-        <v>2307.6923076923076</v>
-      </c>
-      <c r="E5" s="27">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E5" s="15">
         <f>IF($C$6=0,0,C5/$C$6)</f>
-        <v>0.21527612112614608</v>
-      </c>
-      <c r="F5" s="18">
-        <v>0.25</v>
-      </c>
-      <c r="H5" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="H5" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="I5" s="21">
+      <c r="I5" s="9">
         <f>-Informe_final!F8</f>
-        <v>-15000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="66"/>
-      <c r="B6" s="67" t="s">
+      <c r="A6" s="54"/>
+      <c r="B6" s="55" t="s">
         <v>152</v>
       </c>
-      <c r="C6" s="68">
+      <c r="C6" s="56">
         <f>SUM(C3:C5)</f>
-        <v>69677955.555555552</v>
-      </c>
-      <c r="D6" s="69">
+        <v>0</v>
+      </c>
+      <c r="D6" s="57" t="e">
         <f>C6/SUPUESTOS!$C$4</f>
-        <v>10719.685470085469</v>
-      </c>
-      <c r="E6" s="70">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E6" s="58">
         <f>SUM(F3:F5)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="58">
+        <f>SUM(F3:F5)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I6" s="59" t="e">
+        <f>I2+I3+I4+I5</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="I7" s="60" t="e">
+        <f>IF(I2=0,0,I6/I2)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="84" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="84"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="H8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I8" s="61" t="e">
+        <f>I6/SUPUESTOS!$C$4</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
         <v>1</v>
       </c>
-      <c r="F6" s="70">
-        <f>SUM(F3:F5)</f>
-        <v>1</v>
-      </c>
-      <c r="H6" s="71" t="s">
-        <v>153</v>
-      </c>
-      <c r="I6" s="72">
-        <f>I2+I3+I4+I5</f>
-        <v>18670806.155555561</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H7" s="50" t="s">
-        <v>154</v>
-      </c>
-      <c r="I7" s="73">
-        <f>IF(I2=0,0,I6/I2)</f>
-        <v>0.2113307056482201</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="94" t="s">
-        <v>155</v>
-      </c>
-      <c r="B8" s="94"/>
-      <c r="C8" s="94"/>
-      <c r="D8" s="94"/>
-      <c r="E8" s="94"/>
-      <c r="F8" s="94"/>
-      <c r="H8" s="71" t="s">
-        <v>156</v>
-      </c>
-      <c r="I8" s="74">
-        <f>I6/SUPUESTOS!$C$4</f>
-        <v>2872.4317162393172</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>159</v>
-      </c>
-      <c r="F9" s="28" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
-        <v>1</v>
-      </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="9">
         <f>C3</f>
-        <v>39057955.555555552</v>
-      </c>
-      <c r="D10" s="27">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15">
         <f>F3</f>
-        <v>0.6</v>
-      </c>
-      <c r="E10" s="21">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="e">
         <f>$C$6*SUPUESTOS!$C$5*(F3/$F$6)</f>
-        <v>4180677.3333333335</v>
-      </c>
-      <c r="F10" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F10" s="62" t="e">
         <f>E10/SUPUESTOS!$C$4</f>
-        <v>643.18112820512818</v>
-      </c>
-      <c r="H10" s="4" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" s="85" t="s">
         <v>162</v>
       </c>
-      <c r="I10" s="4"/>
+      <c r="I10" s="85"/>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="20">
+      <c r="A11" s="8">
         <v>2</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="9">
         <f>C4</f>
-        <v>15620000</v>
-      </c>
-      <c r="D11" s="27">
+        <v>0</v>
+      </c>
+      <c r="D11" s="15">
         <f>F4</f>
-        <v>0.15</v>
-      </c>
-      <c r="E11" s="21">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="e">
         <f>$C$6*SUPUESTOS!$C$5*(F4/$F$6)</f>
-        <v>1045169.3333333334</v>
-      </c>
-      <c r="F11" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F11" s="62" t="e">
         <f>E11/SUPUESTOS!$C$4</f>
-        <v>160.79528205128204</v>
-      </c>
-      <c r="H11" s="20" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="I11" s="76">
+      <c r="I11" s="63" t="e">
         <f>D22/SUPUESTOS!C20</f>
-        <v>6.7960585931623934</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20">
+      <c r="A12" s="8">
         <v>3</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="9">
         <f>C5</f>
-        <v>15000000</v>
-      </c>
-      <c r="D12" s="27">
+        <v>0</v>
+      </c>
+      <c r="D12" s="15">
         <f>F5</f>
-        <v>0.25</v>
-      </c>
-      <c r="E12" s="21">
-        <v>0</v>
-      </c>
-      <c r="F12" s="75">
+        <v>0</v>
+      </c>
+      <c r="E12" s="9">
+        <v>0</v>
+      </c>
+      <c r="F12" s="62" t="e">
         <f>E12/SUPUESTOS!$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="20" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="I12" s="76">
+      <c r="I12" s="63" t="e">
         <f>D22/SUPUESTOS!C13</f>
-        <v>1235.6470169386171</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="66"/>
-      <c r="B13" s="67" t="s">
+      <c r="A13" s="54"/>
+      <c r="B13" s="55" t="s">
         <v>167</v>
       </c>
-      <c r="C13" s="68">
+      <c r="C13" s="56">
         <f>C6</f>
-        <v>69677955.555555552</v>
-      </c>
-      <c r="D13" s="70">
+        <v>0</v>
+      </c>
+      <c r="D13" s="58">
         <f>SUM(D10:D12)</f>
-        <v>1</v>
-      </c>
-      <c r="E13" s="68">
+        <v>0</v>
+      </c>
+      <c r="E13" s="56" t="e">
         <f>SUM(E10:E12)</f>
-        <v>5225846.666666667</v>
-      </c>
-      <c r="F13" s="69">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F13" s="57" t="e">
         <f>E13/SUPUESTOS!$C$4</f>
-        <v>803.9764102564103</v>
-      </c>
-      <c r="H13" s="20" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="I13" s="76">
+      <c r="I13" s="63" t="e">
         <f>D22/SUPUESTOS!C19</f>
-        <v>308.91175423465427</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H14" s="20" t="s">
+      <c r="H14" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="I14" s="76">
+      <c r="I14" s="63" t="e">
         <f>Laboratorio!G10/SUPUESTOS!C19</f>
-        <v>54.615384615384613</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="I15" s="77">
+      <c r="I15" s="64">
         <f>SUPUESTOS!C21</f>
-        <v>181.81818181818181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="86" t="s">
         <v>171</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
+      <c r="B16" s="86"/>
+      <c r="C16" s="86"/>
+      <c r="D16" s="86"/>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="9">
         <f>C6</f>
-        <v>69677955.555555552</v>
-      </c>
-      <c r="D17" s="75">
+        <v>0</v>
+      </c>
+      <c r="D17" s="62" t="e">
         <f>C17/SUPUESTOS!$C$4</f>
-        <v>10719.685470085469</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="9" t="e">
         <f>E13</f>
-        <v>5225846.666666667</v>
-      </c>
-      <c r="D18" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D18" s="62" t="e">
         <f>C18/SUPUESTOS!$C$4</f>
-        <v>803.9764102564103</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="C19" s="21">
+      <c r="C19" s="9" t="e">
         <f>C17+C18</f>
-        <v>74903802.222222224</v>
-      </c>
-      <c r="D19" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D19" s="62" t="e">
         <f>C19/SUPUESTOS!$C$4</f>
-        <v>11523.661880341881</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="20" t="str">
+      <c r="B20" s="8" t="str">
         <f>CONCATENATE("Retención IVA (",TEXT(SUPUESTOS!C6,"0%"),")")</f>
-        <v>Retención IVA (7%)</v>
-      </c>
-      <c r="C20" s="21">
+        <v>Retención IVA (0%)</v>
+      </c>
+      <c r="C20" s="9" t="e">
         <f>C19*SUPUESTOS!C6</f>
-        <v>5243266.1555555565</v>
-      </c>
-      <c r="D20" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D20" s="62" t="e">
         <f>C20/SUPUESTOS!$C$4</f>
-        <v>806.65633162393181</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="82" t="s">
         <v>240</v>
       </c>
-      <c r="C21" s="97">
+      <c r="C21" s="83">
         <f>+SUM(C3:C4)*0.15</f>
-        <v>8201693.3333333321</v>
-      </c>
-      <c r="D21" s="75">
+        <v>0</v>
+      </c>
+      <c r="D21" s="62" t="e">
         <f>C21/SUPUESTOS!$C$4</f>
-        <v>1261.7989743589742</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="78"/>
-      <c r="B22" s="78" t="s">
+      <c r="A22" s="65"/>
+      <c r="B22" s="65" t="s">
         <v>175</v>
       </c>
-      <c r="C22" s="79">
+      <c r="C22" s="66" t="e">
         <f>C19+C20+C21</f>
-        <v>88348761.711111113</v>
-      </c>
-      <c r="D22" s="80">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D22" s="67" t="e">
         <f>C22/SUPUESTOS!$C$4</f>
-        <v>13592.117186324787</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="68" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="82">
+      <c r="D23" s="69" t="e">
         <f>ROUNDUP(D22,-2)</f>
-        <v>13600</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="94" t="s">
+      <c r="A26" s="84" t="s">
         <v>177</v>
       </c>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="84"/>
     </row>
     <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="95"/>
-      <c r="B27" s="95" t="s">
+      <c r="A27" s="81"/>
+      <c r="B27" s="81" t="s">
         <v>178</v>
       </c>
-      <c r="C27" s="95" t="s">
+      <c r="C27" s="81" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="95" t="s">
+      <c r="D27" s="81" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="B28" s="83" t="s">
+      <c r="B28" s="70" t="s">
         <v>182</v>
       </c>
-      <c r="C28" s="21">
+      <c r="C28" s="9" t="e">
         <f>C3+E10+C21+(C3+E10)/$C$19*C20</f>
-        <v>54467030.524444446</v>
-      </c>
-      <c r="D28" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D28" s="62" t="e">
         <f>ROUNDUP(C28/SUPUESTOS!$C$4,-2)</f>
-        <v>8400</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B29" s="83" t="s">
+      <c r="B29" s="70" t="s">
         <v>184</v>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="9" t="e">
         <f>C4+E11+(C4+E11)/$C$19*C20</f>
-        <v>17831731.186666667</v>
-      </c>
-      <c r="D29" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D29" s="62" t="e">
         <f>ROUNDUP(C29/SUPUESTOS!$C$4,-2)</f>
-        <v>2800</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B30" s="83" t="s">
+      <c r="B30" s="70" t="s">
         <v>186</v>
       </c>
-      <c r="C30" s="21">
+      <c r="C30" s="9" t="e">
         <f>C5+E12+(C5+E12)/$C$19*C20</f>
-        <v>16050000</v>
-      </c>
-      <c r="D30" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D30" s="62" t="e">
         <f>ROUNDUP(C30/SUPUESTOS!$C$4,-2)</f>
-        <v>2500</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="66"/>
-      <c r="B31" s="67" t="s">
+      <c r="A31" s="54"/>
+      <c r="B31" s="55" t="s">
         <v>187</v>
       </c>
-      <c r="C31" s="68">
+      <c r="C31" s="56" t="e">
         <f>SUM(C28:C30)</f>
-        <v>88348761.711111113</v>
-      </c>
-      <c r="D31" s="69">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D31" s="57" t="e">
         <f>+SUM(D28:D30)</f>
-        <v>13700</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -3643,338 +3493,338 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
     </row>
     <row r="3" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="16"/>
+      <c r="B3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="16" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="95" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="84">
+      <c r="C5" s="71">
         <f>SUPUESTOS!C7</f>
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="84">
+        <v>0</v>
+      </c>
+      <c r="D5" s="71">
         <f>SUPUESTOS!C8</f>
-        <v>0.5</v>
-      </c>
-      <c r="E5" s="85">
+        <v>0</v>
+      </c>
+      <c r="E5" s="72">
         <f>C5+D5</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="81" t="s">
+      <c r="B6" s="68" t="s">
         <v>194</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="9" t="e">
         <f>Resumen!C22*C5</f>
-        <v>44174380.855555557</v>
-      </c>
-      <c r="D6" s="21">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D6" s="9" t="e">
         <f>Resumen!C22*D5</f>
-        <v>44174380.855555557</v>
-      </c>
-      <c r="E6" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E6" s="10" t="e">
         <f>C6+D6</f>
-        <v>88348761.711111113</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="C7" s="75">
+      <c r="C7" s="62" t="e">
         <f>C6/SUPUESTOS!$C$4</f>
-        <v>6796.0585931623937</v>
-      </c>
-      <c r="D7" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D7" s="62" t="e">
         <f>D6/SUPUESTOS!$C$4</f>
-        <v>6796.0585931623937</v>
-      </c>
-      <c r="E7" s="75">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E7" s="62" t="e">
         <f>E6/SUPUESTOS!$C$4</f>
-        <v>13592.117186324787</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="96" t="s">
         <v>196</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="B9" s="96"/>
+      <c r="C9" s="96"/>
+      <c r="D9" s="96"/>
+      <c r="E9" s="96"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="64">
+      <c r="C10" s="52">
         <f>Preparación_campo!H12</f>
-        <v>24700000</v>
-      </c>
-      <c r="D10" s="21">
-        <v>0</v>
-      </c>
-      <c r="E10" s="21">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9">
         <f t="shared" ref="E10:E16" si="0">C10+D10</f>
-        <v>24700000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="64">
+      <c r="C11" s="52">
         <f>Preparación_campo!H16</f>
-        <v>7534400</v>
-      </c>
-      <c r="D11" s="21">
-        <v>0</v>
-      </c>
-      <c r="E11" s="21">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9">
         <f t="shared" si="0"/>
-        <v>7534400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C12" s="64">
+      <c r="C12" s="52">
         <f>Preparación_campo!H20</f>
-        <v>4000000</v>
-      </c>
-      <c r="D12" s="21">
-        <v>0</v>
-      </c>
-      <c r="E12" s="21">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0</v>
+      </c>
+      <c r="E12" s="9">
         <f t="shared" si="0"/>
-        <v>4000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="C13" s="64">
+      <c r="C13" s="52">
         <f>Preparación_campo!H27</f>
-        <v>2163555.5555555555</v>
-      </c>
-      <c r="D13" s="21">
-        <v>0</v>
-      </c>
-      <c r="E13" s="21">
+        <v>0</v>
+      </c>
+      <c r="D13" s="9">
+        <v>0</v>
+      </c>
+      <c r="E13" s="9">
         <f t="shared" si="0"/>
-        <v>2163555.5555555555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="C14" s="64">
+      <c r="C14" s="52">
         <f>Preparación_campo!H33</f>
-        <v>660000</v>
-      </c>
-      <c r="D14" s="21">
-        <v>0</v>
-      </c>
-      <c r="E14" s="21">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0</v>
+      </c>
+      <c r="E14" s="9">
         <f t="shared" si="0"/>
-        <v>660000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C15" s="64">
+      <c r="C15" s="52">
         <f>Laboratorio!F10</f>
-        <v>15620000</v>
-      </c>
-      <c r="D15" s="21">
-        <v>0</v>
-      </c>
-      <c r="E15" s="21">
+        <v>0</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0</v>
+      </c>
+      <c r="E15" s="9">
         <f t="shared" si="0"/>
-        <v>15620000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="21">
-        <v>0</v>
-      </c>
-      <c r="D16" s="64">
+      <c r="C16" s="9">
+        <v>0</v>
+      </c>
+      <c r="D16" s="52">
         <f>Informe_final!F8</f>
-        <v>15000000</v>
-      </c>
-      <c r="E16" s="21">
+        <v>0</v>
+      </c>
+      <c r="E16" s="9">
         <f t="shared" si="0"/>
-        <v>15000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="66"/>
-      <c r="B18" s="67" t="s">
+      <c r="A18" s="54"/>
+      <c r="B18" s="55" t="s">
         <v>203</v>
       </c>
-      <c r="C18" s="68">
+      <c r="C18" s="56">
         <f>SUM(C10:C16)</f>
-        <v>54677955.555555552</v>
-      </c>
-      <c r="D18" s="68">
+        <v>0</v>
+      </c>
+      <c r="D18" s="56">
         <f>SUM(D10:D16)</f>
-        <v>15000000</v>
-      </c>
-      <c r="E18" s="68">
+        <v>0</v>
+      </c>
+      <c r="E18" s="56">
         <f>C18+D18</f>
-        <v>69677955.555555552</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="95" t="s">
         <v>204</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+      <c r="B20" s="95"/>
+      <c r="C20" s="95"/>
+      <c r="D20" s="95"/>
+      <c r="E20" s="95"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="81" t="s">
+      <c r="B21" s="68" t="s">
         <v>205</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="10" t="e">
         <f>C6-C18</f>
-        <v>-10503574.699999996</v>
-      </c>
-      <c r="D21" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D21" s="10" t="e">
         <f>D6-D18</f>
-        <v>29174380.855555557</v>
-      </c>
-      <c r="E21" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E21" s="10" t="e">
         <f>C21+D21</f>
-        <v>18670806.155555561</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="81" t="s">
+      <c r="B22" s="68" t="s">
         <v>206</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="10" t="e">
         <f>C21</f>
-        <v>-10503574.699999996</v>
-      </c>
-      <c r="D22" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D22" s="10" t="e">
         <f>C22+D21</f>
-        <v>18670806.155555561</v>
-      </c>
-      <c r="E22" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E22" s="10" t="e">
         <f>D22</f>
-        <v>18670806.155555561</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="68" t="s">
         <v>207</v>
       </c>
-      <c r="C23" s="76">
+      <c r="C23" s="63" t="e">
         <f>C22/SUPUESTOS!$C$4</f>
-        <v>-1615.9345692307686</v>
-      </c>
-      <c r="D23" s="76">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D23" s="63" t="e">
         <f>D22/SUPUESTOS!$C$4</f>
-        <v>2872.4317162393172</v>
-      </c>
-      <c r="E23" s="76">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E23" s="63" t="e">
         <f>E22/SUPUESTOS!$C$4</f>
-        <v>2872.4317162393172</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="97" t="s">
         <v>208</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="B25" s="97"/>
+      <c r="C25" s="97"/>
+      <c r="D25" s="97"/>
+      <c r="E25" s="97"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B26" s="81" t="s">
+      <c r="B26" s="68" t="s">
         <v>209</v>
       </c>
-      <c r="C26" s="86">
+      <c r="C26" s="73" t="e">
         <f>MIN(C22,D22,0)</f>
-        <v>-10503574.699999996</v>
-      </c>
-      <c r="D26" s="17" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="68" t="s">
         <v>211</v>
       </c>
-      <c r="C27" s="87">
+      <c r="C27" s="74" t="e">
         <f>C26/SUPUESTOS!$C$4</f>
-        <v>-1615.9345692307686</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="C28" s="88">
+      <c r="C28" s="75" t="e">
         <f>D22</f>
-        <v>18670806.155555561</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="B30" s="71" t="s">
+      <c r="B30" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C30" s="89">
+      <c r="C30" s="76" t="e">
         <f>E22</f>
-        <v>18670806.155555561</v>
-      </c>
-      <c r="D30" s="90">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D30" s="77" t="e">
         <f>C30/SUPUESTOS!$C$4</f>
-        <v>2872.4317162393172</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -4006,92 +3856,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="16" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="16">
-        <v>6240000</v>
-      </c>
-      <c r="D2" s="91">
-        <v>60</v>
-      </c>
-      <c r="E2" s="21">
+      <c r="C2" s="5"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="9">
         <f>IF(D2=0,0,C2/D2)</f>
-        <v>104000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20">
+      <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="16">
-        <v>8000000</v>
-      </c>
-      <c r="D3" s="91">
-        <v>60</v>
-      </c>
-      <c r="E3" s="21">
+      <c r="C3" s="5"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="9">
         <f>IF(D3=0,0,C3/D3)</f>
-        <v>133333.33333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="16">
-        <v>3000000</v>
-      </c>
-      <c r="D4" s="91">
-        <v>60</v>
-      </c>
-      <c r="E4" s="21">
+      <c r="C4" s="5"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="9">
         <f>IF(D4=0,0,C4/D4)</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="8">
         <v>4</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="16">
-        <v>2200000</v>
-      </c>
-      <c r="D5" s="91">
-        <v>36</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="C5" s="5"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="9">
         <f>IF(D5=0,0,C5/D5)</f>
-        <v>61111.111111111109</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4115,104 +3949,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="16" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="C2" s="16">
-        <v>10</v>
-      </c>
-      <c r="D2" s="16">
-        <v>20000</v>
-      </c>
-      <c r="E2" s="21">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="9">
         <f>C2*D2</f>
-        <v>200000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20">
+      <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="C3" s="16">
-        <v>10</v>
-      </c>
-      <c r="D3" s="16">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="21">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="9">
         <f>C3*D3</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C4" s="16">
-        <v>1</v>
-      </c>
-      <c r="D4" s="16">
-        <v>80000</v>
-      </c>
-      <c r="E4" s="21">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="9">
         <f>C4*D4</f>
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="8">
         <v>4</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="C5" s="16">
-        <v>1</v>
-      </c>
-      <c r="D5" s="16">
-        <v>50000</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="9">
         <f>C5*D5</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="92"/>
-      <c r="B6" s="92" t="s">
+      <c r="A6" s="79"/>
+      <c r="B6" s="79" t="s">
         <v>191</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="93">
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="80">
         <f>SUM(E2:E5)</f>
-        <v>380000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>